<commit_message>
modify default string comparison behavior, now is case insensitive. Add new system parameter: $StrCompareCaseSensitive=true
</commit_message>
<xml_diff>
--- a/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/IfACellEqString.xlsx
+++ b/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/IfACellEqString.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/Lexerow/Dev/Lexerow/2-Tests/Lexerow.Core.Tests/10-Files/Run/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/Lexerow/Dev/Lexerow/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_2B8C63A238C272CACCFC3B895DC533011B7D74F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2570602A-1E3A-4365-A330-A05B0E2F95CE}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_2B8C63A238C272CACCFC3B895DC533011B7D74F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{247D92DD-9F32-4630-A161-F3D2BC076F91}"/>
   <bookViews>
-    <workbookView xWindow="6150" yWindow="1785" windowWidth="18720" windowHeight="12330" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10125" yWindow="7425" windowWidth="16380" windowHeight="9735" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
   <si>
     <t>Hello</t>
   </si>
@@ -37,6 +37,21 @@
   </si>
   <si>
     <t>colA</t>
+  </si>
+  <si>
+    <t>If A.Cell="Hello" Then A.Cell="Bonjour"</t>
+  </si>
+  <si>
+    <t>expected</t>
+  </si>
+  <si>
+    <t>Bonjour</t>
+  </si>
+  <si>
+    <t>HELLO</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -55,12 +70,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -75,9 +96,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -93,6 +115,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -358,31 +384,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>